<commit_message>
data: add Andal Sindhu (andal.sindhu@accenture.com, dob 16/09/1991)
</commit_message>
<xml_diff>
--- a/employees.xlsx
+++ b/employees.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,6 +591,48 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Andal Sindhu</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>andal.sindhu</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>andal.sindhu@accenture.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>16/09/1991</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Mapla, Antigravity</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>antigravitymapla@gmail.com</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>

</xml_diff>